<commit_message>
R2.8: columnas HSS 10x10x1/2 en el peso propio y W = 17.49 t en sismo; documentos de parámetros y densidad basados en las hojas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ns7QgNzAi3QoiHRE1oS8iD
</commit_message>
<xml_diff>
--- a/AreasTributarias_NOSE_DOCK_H5_H6_R2.8.xlsx
+++ b/AreasTributarias_NOSE_DOCK_H5_H6_R2.8.xlsx
@@ -13822,18 +13822,18 @@
     <row r="23">
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>HSST10X10X0.313</t>
+          <t>HSST10X10X0.5</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
         <v>59.88</v>
       </c>
-      <c r="D23" s="29" t="n">
-        <v>69.6773</v>
+      <c r="D23" s="29">
+        <v>110.9675</v>
       </c>
       <c r="E23" s="18">
         <f>C23*100*D23*0.00783341</f>
-        <v>3268.31542125488</v>
+        <v>5205.0924979599</v>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
@@ -13986,7 +13986,7 @@
       <c r="D30" s="7" t="n"/>
       <c r="E30" s="18">
         <f>SUM(E23:E29)</f>
-        <v>9884.72253574939</v>
+        <v>11821.4996124544</v>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
@@ -14036,7 +14036,7 @@
       </c>
       <c r="C34" s="10">
         <f>E30/1000</f>
-        <v>9.88472253574939</v>
+        <v>11.8214996124544</v>
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
@@ -14166,7 +14166,7 @@
       </c>
       <c r="C39" s="10">
         <f>SUM(C34:C38)</f>
-        <v>15.5517241137494</v>
+        <v>17.4885011904544</v>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
@@ -14192,7 +14192,7 @@
       </c>
       <c r="C40" s="14" t="str">
         <f>"La suma de cargas del caso 1 debe dar ≈ "&amp;TEXT(C34+C35+C36+C37,"0.00")&amp;" t"</f>
-        <v>La suma de cargas del caso 1 debe dar ≈ 15.55 t</v>
+        <v>La suma de cargas del caso 1 debe dar ≈ 17.49 t</v>
       </c>
       <c r="D40" s="7" t="inlineStr"/>
       <c r="E40" s="8" t="inlineStr">

</xml_diff>